<commit_message>
Add index-check skill and update positions to extended version
</commit_message>
<xml_diff>
--- a/data/positions/output.xlsx
+++ b/data/positions/output.xlsx
@@ -460,16 +460,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://lemanapro.ru/catalogue/gotovye-okna/</t>
+          <t>https://lemanapro.ru/catalogue/plastikovye-okna/</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-14</t>
         </is>
       </c>
     </row>
@@ -484,12 +484,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://lemanapro.ru/catalogue/plastikovye-okna/v-kvartiru/</t>
+          <t>https://lemanapro.ru/catalogue/plastikovye-okna/</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-14</t>
         </is>
       </c>
     </row>
@@ -504,12 +504,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://lemanapro.ru/catalogue/gotovye-okna/</t>
+          <t>https://lemanapro.ru/catalogue/plastikovye-okna/</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-14</t>
         </is>
       </c>
     </row>
@@ -520,16 +520,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://lemanapro.ru/catalogue/plastikovye-okna/v-kvartiru/</t>
+          <t>https://lemanapro.ru/catalogue/plastikovye-okna/</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-14</t>
         </is>
       </c>
     </row>
@@ -544,12 +544,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://lemanapro.ru/catalogue/gotovye-okna/</t>
+          <t>https://lemanapro.ru/catalogue/plastikovye-okna/</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-14</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -569,7 +569,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-14</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -625,7 +625,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-14</t>
         </is>
       </c>
     </row>
@@ -636,16 +636,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://nizhniy-novgorod.lemanapro.ru/catalogue/plastikovye-okna/</t>
+          <t>https://lemanapro.ru/catalogue/plastikovye-okna/</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-14</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-14</t>
         </is>
       </c>
     </row>
@@ -672,7 +672,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -681,7 +681,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-14</t>
         </is>
       </c>
     </row>
@@ -692,7 +692,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -701,7 +701,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-14</t>
         </is>
       </c>
     </row>
@@ -712,16 +712,12 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>25</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>https://nizhniy-novgorod.lemanapro.ru/catalogue/plastikovye-okna/rehau/</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-14</t>
         </is>
       </c>
     </row>
@@ -804,7 +800,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.mosokna.ru/plastikovye-okna</t>
+          <t>https://www.mosokna.ru/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -814,12 +810,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://shop.oknagorizont.ru/catalog/gotovye-plastikovye-okna-pvh-so-sklada/</t>
+          <t>https://moscow.petrovich.ru/catalog/15635/</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://oknalux.ru/catalog/plastikovye_okna/</t>
+          <t>https://www.ozon.ru/category/plastikovye-okna-34491/</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -829,27 +825,27 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.plastika-okon.ru/</t>
+          <t>https://xn-----6kccad2akgz2afhej9d.xn--p1ai/</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://moscow.petrovich.ru/catalog/15635/</t>
+          <t>https://oknavigoda.ru/catalog/plastikovye-okna/</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://xn-----6kccad2akgz2afhej9d.xn--p1ai/plastikovie-okna/okna-v-kvartiru</t>
+          <t>https://www.plastika-okon.ru/okna/</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>https://www.okna-proizvodstvo.ru/</t>
+          <t>https://www.msk.okna-servise.com/plastikovye-okna/gotovye-okna/?page=3</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://www.fabrikaokon.ru/okna.html</t>
+          <t>https://23okna.ru/</t>
         </is>
       </c>
     </row>
@@ -861,17 +857,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>https://xn-----6kccad2akgz2afhej9d.xn--p1ai/plastikovie-okna</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>https://www.mosokna.ru/</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>https://xn-----6kccad2akgz2afhej9d.xn--p1ai/plastikovie-okna</t>
-        </is>
-      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://lemanapro.ru/catalogue/gotovye-okna/</t>
+          <t>https://lemanapro.ru/catalogue/plastikovye-okna/</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -886,27 +882,27 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
+          <t>https://www.ramokna.ru/okna-plastikovyie/</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
           <t>https://www.ozon.ru/category/plastikovye-okna-34491/</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>https://www.ramokna.ru/okna-plastikovyie/</t>
-        </is>
-      </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>https://oknalux.ru/catalog/plastikovye_okna/</t>
+          <t>https://oknavigoda.ru/catalog/plastikovye-okna/</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://oknavigoda.ru/catalog/plastikovye-okna/</t>
+          <t>https://www.okna-moskva.ru/</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>https://www.okna-moskva.ru/gotovye-plastikovye-okna/</t>
+          <t>https://online-shop.rhsolutions.ru/products/plastikovoe-okno-pvh-rehau-ehperience-grazio-profil-70-mm-1200h700-mm-vhsh-s-uchetom-podstavochnogo-profilya-odnostvorchatoe-gluhoe-energosberegay-264467</t>
         </is>
       </c>
     </row>
@@ -928,12 +924,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://lemanapro.ru/catalogue/gotovye-okna/</t>
+          <t>https://lemanapro.ru/catalogue/plastikovye-okna/</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://shop.oknagorizont.ru/catalog/gotovye-plastikovye-okna-pvh-so-sklada/</t>
+          <t>https://moscow.petrovich.ru/catalog/15635/</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -943,27 +939,27 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://oknalux.ru/catalog/plastikovye_okna/</t>
+          <t>https://www.okna-moskva.ru/</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://moscow.petrovich.ru/catalog/15635/</t>
+          <t>https://www.ramokna.ru/okna-plastikovyie/</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>https://www.okna-moskva.ru/gotovye-plastikovye-okna/</t>
+          <t>https://oknavigoda.ru/catalog/plastikovye-okna/</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>https://www.ramokna.ru/kalkulyator-okon/</t>
+          <t>https://www.ozon.ru/category/plastikovye-okna-34491/</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>https://online-shop.rhsolutions.ru/products/plastikovoe-okno-pvh-rehau-ehperience-blitz-1440h870-mm-vhsh-s-uchetom-podstavochnogo-profilya-odnostvorchatoe-povorotno-otkidnoe-levoe-dvuhkamern-3-264837</t>
+          <t>https://yandex.ru/images/search?text=%D0%BE%D0%BA%D0%BD%D0%B0+%D0%BF%D0%B2%D1%85+%D0%BC%D0%BE%D1%81%D0%BA%D0%B2%D0%B0</t>
         </is>
       </c>
     </row>
@@ -975,52 +971,52 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.mosokna.ru/plastikovye-okna/vidy-okon/dvuhstvorchatoe-okno</t>
+          <t>https://www.mosokna.ru/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://xn-----6kccad2akgz2afhej9d.xn--p1ai/plastikovie-okna</t>
+          <t>https://lemanapro.ru/catalogue/plastikovye-okna/v-kvartiru/</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
+          <t>https://moscow.petrovich.ru/catalog/15635/</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
           <t>https://www.plastika-okon.ru/</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://shop.oknagorizont.ru/catalog/gotovye-plastikovye-okna-pvh-so-sklada/</t>
-        </is>
-      </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://lemanapro.ru/catalogue/plastikovye-okna/v-kvartiru/</t>
+          <t>https://xn-----6kccad2akgz2afhej9d.xn--p1ai/</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
+          <t>https://oknavigoda.ru/catalog/plastikovye-okna/</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>https://www.okna-moskva.ru/gotovye-plastikovye-okna/</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>https://www.ramokna.ru/okna-plastikovyie/</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
           <t>https://oknalux.ru/catalog/plastikovye_okna/</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>https://www.ramokna.ru/okna-plastikovyie/</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>https://moscow.petrovich.ru/catalog/15635/</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>https://www.msk.okna-servise.com/plastikovye-okna/gotovye-okna/?page=3</t>
-        </is>
-      </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>https://www.okna-moskva.ru/prices/</t>
+          <t>https://www.msk.okna-servise.com/plastikovye-okna/gotovye-okna/</t>
         </is>
       </c>
     </row>
@@ -1032,12 +1028,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.mosokna.ru/</t>
+          <t>https://www.mosokna.ru/ceny/rassrochka</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://lemanapro.ru/catalogue/gotovye-okna/</t>
+          <t>https://lemanapro.ru/catalogue/plastikovye-okna/</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1047,14 +1043,14 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>https://shop.oknagorizont.ru/catalog/gotovye-plastikovye-okna-pvh-so-sklada/</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>https://moscow.petrovich.ru/catalog/15635/</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>https://shop.oknagorizont.ru/</t>
-        </is>
-      </c>
       <c r="G6" t="inlineStr">
         <is>
           <t>https://www.ozon.ru/category/plastikovye-okna-34491/</t>
@@ -1072,12 +1068,12 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>https://oknalux.ru/catalog/plastikovye_okna/</t>
+          <t>https://www.plastika-okon.ru/</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>https://www.plastika-okon.ru/</t>
+          <t>https://oknavigoda.ru/catalog/plastikovye-okna/</t>
         </is>
       </c>
     </row>
@@ -1089,42 +1085,42 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>https://xn-----6kccad2akgz2afhej9d.xn--p1ai/plastikovie-okna/rehau</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://fabrikauyuta.ru/rehau-okna/</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
           <t>https://rhsolutions.ru/</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>https://www.mosokna.ru/plastikovye-okna-rehau</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>https://fabrikauyuta.ru/rehau-okna/</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>https://lemanapro.ru/catalogue/plastikovye-okna/rehau/</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>https://xn-----6kccad2akgz2afhej9d.xn--p1ai/plastikovie-okna/rehau</t>
-        </is>
-      </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.ramokna.ru/plastikovyie-okna-rehau/</t>
+          <t>https://www.ozon.ru/category/plastikovye-okna-34491/rehau-87247520/</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
+          <t>https://www.ramokna.ru/calculator-rehau/</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
           <t>https://i-okna.ru/okna/blitz</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>https://www.okna-moskva.ru/plastikovye-okna-rehau/</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1237,14 +1233,14 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>https://mosdvery.ru/categories/okna-plastikovye</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
           <t>https://oknafactoria.ru/gotovie-okna/</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>https://mosdvery.ru/categories/okna-plastikovye</t>
-        </is>
-      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>https://inokna.by/stati/36-kak-vybrat-okno-pvkh-nashi-rekomendatsii.html</t>
@@ -1252,7 +1248,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://okno-msk.ru/</t>
+          <t>https://2gis.ru/moscow/search/%D0%9F%D0%B2%D1%85%20%D0%BE%D0%BA%D0%BD%D0%B0</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -1262,7 +1258,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://2gis.ru/moscow/search/%D0%9F%D0%BB%D0%B0%D1%81%D1%82%D0%B8%D0%BA%D0%BE%D0%B2%D1%8B%D0%B5%20%D0%BE%D0%BA%D0%BD%D0%B0</t>
+          <t>https://23okna.ru/plastikovye-okna/</t>
         </is>
       </c>
     </row>
@@ -1274,52 +1270,52 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://okno.ru/</t>
+          <t>https://www.oknakomforta.ru/produkcija/plastikovye-okna/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.eurookna.ru/plastikovye-okna/</t>
+          <t>https://okonti.ru/</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://okno-msk.ru/</t>
+          <t>https://www.design-okno.ru/</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.oknakomforta.ru/produkcija/plastikovye-okna/</t>
+          <t>https://okno.ru/okna-rehau/plastikovye-okna-pod-klyuch/</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.oknastreet.ru/stoimost-new/plastikovye-okna-ceny.html</t>
+          <t>https://kostroma.oknamydom.ru/plastikovie-okna/</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.fabrikaokon.ru/okna.html</t>
+          <t>https://kazan.vsevdom.info/windows/windows</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://2gis.ru/moscow/search/%D0%9F%D0%BB%D0%B0%D1%81%D1%82%D0%B8%D0%BA%D0%BE%D0%B2%D1%8B%D0%B5%20%D0%BE%D0%BA%D0%BD%D0%B0</t>
+          <t>https://tp-okna.ru/plastikovye-okna/</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>https://www.oknaprosvet.ru/okna-ceny/</t>
+          <t>https://www.veka.ru/calc</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://okno.ru/okna-rehau/plastikovye-okna-pod-klyuch/</t>
+          <t>https://красноярск.надежныеокна.рф/%D1%86%D0%B5%D0%BD%D1%8B</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>https://mosdvery.ru/categories/okna-plastikovye</t>
+          <t>https://www.semokna.ru/plastikovie_okna</t>
         </is>
       </c>
     </row>
@@ -1361,22 +1357,22 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.plastika-okon.ru/</t>
+          <t>https://okno-msk.ru/</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
+          <t>https://www.oknastreet.ru/stoimost-new/plastikovye-okna-ceny.html</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>https://www.oknastar.ru/rasprodazha-gotovykh-pvkh-okon/</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
           <t>https://www.mosokna.ru/</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>https://www.oknastar.ru/rasprodazha-gotovykh-pvkh-okon/</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>https://www.oknastreet.ru/stoimost-new/plastikovye-okna-ceny.html</t>
         </is>
       </c>
     </row>
@@ -1428,12 +1424,12 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>https://www.oknastar.ru/rasprodazha-gotovykh-pvkh-okon/</t>
+          <t>https://rusokna.ru/ceny/</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>https://rusokna.ru/ceny/</t>
+          <t>https://www.okna-proizvodstvo.ru/</t>
         </is>
       </c>
     </row>
@@ -1445,29 +1441,29 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>https://okno.ru/</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>https://www.oknakomforta.ru/produkcija/plastikovye-okna/</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>https://www.eurookna.ru/plastikovye-okna/</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>https://okno.ru/</t>
-        </is>
-      </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>https://www.fabrikaokon.ru/okna.html</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>https://www.okna.ru/dizajnerskie-okna/</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>https://www.oknaprosvet.ru/okna-ceny/</t>
-        </is>
-      </c>
       <c r="G6" t="inlineStr">
         <is>
           <t>https://www.mosokna.ru/</t>
@@ -1475,22 +1471,22 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
+          <t>https://www.oknastar.ru/rasprodazha-gotovykh-pvkh-okon/</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>https://www.oknaprosvet.ru/</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>https://okno-msk.ru/</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
           <t>https://www.plastika-okon.ru/</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>https://www.veka.ru/production/plastikovye-okna/prostoe-okno</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>https://okno-msk.ru/</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>https://www.fabrikaokon.ru/okna.html</t>
         </is>
       </c>
     </row>
@@ -1507,14 +1503,14 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
+          <t>https://www.oknaprosvet.ru/okna-rehau/</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
           <t>https://okno.ru/okna-rehau/podmoskove/moskovskij/</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>https://www.oknaprosvet.ru/okna-rehau/</t>
-        </is>
-      </c>
       <c r="E7" t="inlineStr">
         <is>
           <t>https://rhsolutions.ru/</t>
@@ -1527,27 +1523,27 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
+          <t>https://rhsolutions.ru/store/catalog/plastikovie-okna-i-dveri/</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
           <t>https://www.oknastreet.ru/products/plastikovye-okna/rehau.html</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>https://i-okna.ru/</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>https://okna-moscow.ru/plastikovye-okna/rehau/</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
         <is>
           <t>https://www.mosokna.ru/plastikovye-okna-rehau</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>https://okno.ru/okna-rehau/podmoskove/moskovskij/</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>https://www.oknaprosvet.ru/okna-rehau/</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>https://rhsolutions.ru/</t>
         </is>
       </c>
     </row>

</xml_diff>